<commit_message>
menambah pilihan sorter hari
</commit_message>
<xml_diff>
--- a/open_tracker_data.xlsx
+++ b/open_tracker_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,6 +569,68 @@
       <c r="G5" t="inlineStr">
         <is>
           <t>2026-08-06 23:00:21.851479</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>pemasukkan</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>jatah 1 bulan</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Jumat 7 Agustus 2026, 22:13</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-08-07 22:13:05.404660</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>pemasukkan</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>bonus</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Jumat 7 Agustus 2026, 22:13</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-08-07 22:13:50.181600</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
menambahkan keperluan module untuk deploy requirements
</commit_message>
<xml_diff>
--- a/open_tracker_data.xlsx
+++ b/open_tracker_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -634,6 +634,99 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>pemasukkan</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>tip</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>150000</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Sabtu 8 Agustus 2026, 21:15</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-08-08 21:15:25.024642</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>pengeluaran</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>beras 10kg</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>250000</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Sabtu 8 Agustus 2026, 21:15</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-08-08 21:15:38.889259</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>pengeluaran</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>makan malam</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>225000</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Sabtu 8 Agustus 2026, 21:17</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-08-08 21:17:45.029862</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>